<commit_message>
Preserve team-entered RTM data when regenerating
build_rtm.py now merges with the existing workbook by Req ID: document-
derived columns are refreshed, team-maintained columns (fit-gap, design
ref, test case ID/type/phase, status, defects, owner, notes) are kept,
extra test-case rows are retained as "Additional Test Case", and rows
whose ID left the documents move to an Orphaned sheet. Priority follows
the documents with conflicts reported. Writes a .bak copy and replaces
the file atomically; --fresh starts blank. Summary counts test cases
separately from items. Ignore backup/temp/Excel lock files.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/rtm/AstraWMS_RTM.xlsx
+++ b/docs/rtm/AstraWMS_RTM.xlsx
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -598,265 +598,277 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Maintain only the yellow-header columns on the RTM sheet (Fit-Gap Disposition, Design Reference, Test Status, Defect ID(s), Owner). Summary recalculates automatically. Add further test cases for a requirement as extra rows with the same Req ID and TC suffix -02, -03 …</t>
+          <t>Maintain the yellow-header columns on the RTM sheet (Fit-Gap Disposition, Design Reference, Test Status, Defect ID(s), Owner); Test Case ID, Test Type, Test Phase and Notes may also be edited. Summary recalculates automatically. Add further test cases for a requirement as extra rows with the same Req ID; they are typed 'Additional Test Case' on the next regeneration.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="4" t="n"/>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Regenerating</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>python docs/rtm/build_rtm.py refreshes the document-derived columns (Req ID to Priority) and keeps everything the team entered, matched by Req ID. Priority always follows the scope documents: change it there. Rows whose Req ID was removed from the documents move to the Orphaned sheet. The previous file is saved as AstraWMS_RTM.bak.xlsx. --fresh starts from a blank matrix.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Meaning</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Req ID</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Identifier from the scope documents: &lt;AREA&gt;-&lt;NNN&gt; requirement, &lt;AREA&gt;-EX-&lt;NN&gt; exception flow, IF-&lt;FLOW&gt;-&lt;NNN&gt; ERP interface.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Req ID</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Requirement | Exception | Interface.</t>
+          <t>Identifier from the scope documents: &lt;AREA&gt;-&lt;NNN&gt; requirement, &lt;AREA&gt;-EX-&lt;NN&gt; exception flow, IF-&lt;FLOW&gt;-&lt;NNN&gt; ERP interface.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Area / Section / Source Document</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Functional area (from the ID prefix), the heading it appears under, and the Markdown file that defines it.</t>
+          <t>Requirement | Exception | Interface | Additional Test Case (extra test-case row for a Req ID; excluded from item, priority and fit-gap counts).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Requirement / Exception</t>
+          <t>Area / Section / Source Document</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Requirement text, exception name, or interface object/direction/trigger as written in the scope.</t>
+          <t>Functional area (from the ID prefix), the heading it appears under, and the Markdown file that defines it.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Acceptance Criteria</t>
+          <t>Requirement / Exception</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Rules: enforced as stated (positive + negative case). Exceptions: detection, resolution and ERP impact from the exception table. Interfaces: SAP/Oracle technology, design peak volume and latency SLA. HA/DR NFRs: the stated target.</t>
+          <t>Requirement text, exception name, or interface object/direction/trigger as written in the scope.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Priority</t>
+          <t>Acceptance Criteria</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>MoSCoW: M Must, S Should, C Could, W Won't (document §0.4).</t>
+          <t>Rules: enforced as stated (positive + negative case). Exceptions: detection, resolution and ERP impact from the exception table. Interfaces: SAP/Oracle technology, design peak volume and latency SLA. HA/DR NFRs: the stated target.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Fit-Gap Disposition (input)</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Blueprint outcome (§I.1.2): Fit - Standard, Fit - Configuration, Gap - Extension, Gap - Process Change, Rejected, Deferred.</t>
+          <t>MoSCoW: M Must, S Should, C Could, W Won't (document §0.4).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Design Reference (input)</t>
+          <t>Fit-Gap Disposition (input)</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Process Design Document (PDD) or Interface Specification Document (ISD) reference.</t>
+          <t>Blueprint outcome (§I.1.2): Fit - Standard, Fit - Configuration, Gap - Extension, Gap - Process Change, Rejected, Deferred.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Test Case ID</t>
+          <t>Design Reference (input)</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Generated placeholder TC-&lt;ReqID&gt;-01; replace/extend with IDs from the test management tool.</t>
+          <t>Process Design Document (PDD) or Interface Specification Document (ISD) reference.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Test Type / Test Phase</t>
+          <t>Test Case ID</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Proposed from the Testing Strategy (§I.2): functional, exception, integration, interface, performance, resilience/DR, security &amp; audit, automation, regulated validation.</t>
+          <t>Generated placeholder TC-&lt;ReqID&gt;-01; replace/extend with IDs from the test management tool.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>Test Type / Test Phase</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Proposed from the Testing Strategy (§I.2): functional, exception, integration, interface, performance, resilience/DR, security &amp; audit, automation, regulated validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
           <t>Test Status (input)</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Not Started, In Progress, Passed, Failed, Blocked, Deferred, N/A.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="n"/>
-      <c r="B17" s="4" t="n"/>
-    </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="3" t="n"/>
+      <c r="B18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Example (filled row)</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Req ID INB-002 · Fit-Gap Disposition: Fit - Configuration · Design Reference: PDD-INB-01 §3.2 · Test Status: Passed · Defect ID(s): DEF-0142 (closed) · Owner: Receiving Process Owner</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="n"/>
-      <c r="B19" s="4" t="n"/>
-    </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="3" t="n"/>
+      <c r="B20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Assumptions</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Exception codes carry no priority in the scope; they are set to M because §I.2 requires every exception code to be covered by a test case.</t>
-        </is>
-      </c>
+      <c r="B21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>NFR-020 to NFR-030 (HA/DR) list a target instead of a priority; they are set to M.</t>
+          <t>Exception codes carry no priority in the scope; they are set to M because §I.2 requires every exception code to be covered by a test case.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Interfaces IF-* are set to M; drop to S/C per site if an interface is not used (e.g. kitting IF-KIT-001 at sites without kitting).</t>
+          <t>NFR-020 to NFR-030 (HA/DR) list a target instead of a priority; they are set to M.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Where a priority carries a qualifier (e.g. 'M (if sorter in scope)'), the letter is used and the qualifier is kept in Notes.</t>
+          <t>Interfaces IF-* are set to M; drop to S/C per site if an interface is not used (e.g. kitting IF-KIT-001 at sites without kitting).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Test Type and Phase are proposals derived from the requirement wording (latency/throughput targets → Performance; e-signature/Part 11 → Regulated validation). Confirm during test planning.</t>
+          <t>Where a priority carries a qualifier (e.g. 'M (if sorter in scope)'), the letter is used and the qualifier is kept in Notes.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>KPI and report rows (RPT-*) take the KPI formula, target and grain, or the report frequency, audience and contents, as acceptance criteria. Web UI module rows (UX-*) take the key screens and primary roles.</t>
+          <t>Test Type and Phase are proposals derived from the requirement wording (latency/throughput targets → Performance; e-signature/Part 11 → Regulated validation). Confirm during test planning.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>KPI and report rows (RPT-*) take the KPI formula, target and grain, or the report frequency, audience and contents, as acceptance criteria. Web UI module rows (UX-*) take the key screens and primary roles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
           <t>Coverage</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Traced: every numbered requirement, exception code and interface, plus §D.5 Integration Security (INT-020–027), §E.4 Security &amp; Compliance (NFR-100–109), §E.6 API Governance (NFR-120–129), §G.2 Web UI Modules (UX-001–017), §H.3–H.6 KPIs and reports (RPT-001–070). Not traced as separate rows: descriptive design tables (§F architecture, §D.1–D.4 mappings, §G.3–G.6 RF flows/voice/RBAC/dashboards, §H.7 data warehouse), which are verified through the requirements that reference them.</t>
         </is>
@@ -873,7 +885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O27"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -891,6 +903,7 @@
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -955,30 +968,35 @@
       </c>
       <c r="J4" s="9" t="inlineStr">
         <is>
+          <t>Test Cases</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>Failed / Blocked</t>
         </is>
       </c>
-      <c r="L4" s="9" t="inlineStr">
+      <c r="M4" s="9" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="M4" s="9" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>% Passed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>% Test Cases Passed</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
         <is>
           <t>% Fit-Gap Assessed</t>
         </is>
@@ -991,7 +1009,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A5)</f>
+        <f>C5+D5+E5</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -1007,42 +1025,46 @@
         <v/>
       </c>
       <c r="F5" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A5,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A5,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G5" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A5,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A5,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H5" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A5,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A5,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I5" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A5,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A5,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J5" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A5)</f>
+        <v/>
+      </c>
+      <c r="K5" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A5,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K5" s="11">
+      <c r="L5" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A5,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A5,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L5" s="11">
+      <c r="M5" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A5,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M5" s="11">
+      <c r="N5" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A5,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N5" s="12">
-        <f>IFERROR(J5/B5,0)</f>
-        <v/>
-      </c>
       <c r="O5" s="12">
+        <f>IFERROR(K5/J5,0)</f>
+        <v/>
+      </c>
+      <c r="P5" s="12">
         <f>IFERROR(I5/B5,0)</f>
         <v/>
       </c>
@@ -1054,7 +1076,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A6)</f>
+        <f>C6+D6+E6</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -1070,42 +1092,46 @@
         <v/>
       </c>
       <c r="F6" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A6,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A6,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G6" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A6,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A6,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H6" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A6,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A6,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I6" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A6,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A6,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J6" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A6)</f>
+        <v/>
+      </c>
+      <c r="K6" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A6,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K6" s="11">
+      <c r="L6" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A6,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A6,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L6" s="11">
+      <c r="M6" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A6,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M6" s="11">
+      <c r="N6" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A6,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N6" s="12">
-        <f>IFERROR(J6/B6,0)</f>
-        <v/>
-      </c>
       <c r="O6" s="12">
+        <f>IFERROR(K6/J6,0)</f>
+        <v/>
+      </c>
+      <c r="P6" s="12">
         <f>IFERROR(I6/B6,0)</f>
         <v/>
       </c>
@@ -1117,7 +1143,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A7)</f>
+        <f>C7+D7+E7</f>
         <v/>
       </c>
       <c r="C7" s="11">
@@ -1133,42 +1159,46 @@
         <v/>
       </c>
       <c r="F7" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A7,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A7,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G7" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A7,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A7,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H7" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A7,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A7,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I7" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A7,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A7,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J7" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A7,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K7" s="11">
+      <c r="L7" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A7,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A7,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L7" s="11">
+      <c r="M7" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A7,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M7" s="11">
+      <c r="N7" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A7,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N7" s="12">
-        <f>IFERROR(J7/B7,0)</f>
-        <v/>
-      </c>
       <c r="O7" s="12">
+        <f>IFERROR(K7/J7,0)</f>
+        <v/>
+      </c>
+      <c r="P7" s="12">
         <f>IFERROR(I7/B7,0)</f>
         <v/>
       </c>
@@ -1180,7 +1210,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A8)</f>
+        <f>C8+D8+E8</f>
         <v/>
       </c>
       <c r="C8" s="11">
@@ -1196,42 +1226,46 @@
         <v/>
       </c>
       <c r="F8" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A8,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A8,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G8" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A8,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A8,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H8" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A8,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A8,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I8" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A8,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A8,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J8" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A8,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K8" s="11">
+      <c r="L8" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A8,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A8,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L8" s="11">
+      <c r="M8" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A8,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M8" s="11">
+      <c r="N8" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A8,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N8" s="12">
-        <f>IFERROR(J8/B8,0)</f>
-        <v/>
-      </c>
       <c r="O8" s="12">
+        <f>IFERROR(K8/J8,0)</f>
+        <v/>
+      </c>
+      <c r="P8" s="12">
         <f>IFERROR(I8/B8,0)</f>
         <v/>
       </c>
@@ -1243,7 +1277,7 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A9)</f>
+        <f>C9+D9+E9</f>
         <v/>
       </c>
       <c r="C9" s="11">
@@ -1259,42 +1293,46 @@
         <v/>
       </c>
       <c r="F9" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A9,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A9,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G9" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A9,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A9,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H9" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A9,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A9,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I9" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A9,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A9,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J9" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A9,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K9" s="11">
+      <c r="L9" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A9,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A9,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L9" s="11">
+      <c r="M9" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A9,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M9" s="11">
+      <c r="N9" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A9,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N9" s="12">
-        <f>IFERROR(J9/B9,0)</f>
-        <v/>
-      </c>
       <c r="O9" s="12">
+        <f>IFERROR(K9/J9,0)</f>
+        <v/>
+      </c>
+      <c r="P9" s="12">
         <f>IFERROR(I9/B9,0)</f>
         <v/>
       </c>
@@ -1306,7 +1344,7 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A10)</f>
+        <f>C10+D10+E10</f>
         <v/>
       </c>
       <c r="C10" s="11">
@@ -1322,42 +1360,46 @@
         <v/>
       </c>
       <c r="F10" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A10,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A10,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G10" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A10,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A10,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H10" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A10,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A10,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I10" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A10,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A10,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J10" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A10,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K10" s="11">
+      <c r="L10" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A10,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A10,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L10" s="11">
+      <c r="M10" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A10,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M10" s="11">
+      <c r="N10" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A10,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N10" s="12">
-        <f>IFERROR(J10/B10,0)</f>
-        <v/>
-      </c>
       <c r="O10" s="12">
+        <f>IFERROR(K10/J10,0)</f>
+        <v/>
+      </c>
+      <c r="P10" s="12">
         <f>IFERROR(I10/B10,0)</f>
         <v/>
       </c>
@@ -1369,7 +1411,7 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A11)</f>
+        <f>C11+D11+E11</f>
         <v/>
       </c>
       <c r="C11" s="11">
@@ -1385,42 +1427,46 @@
         <v/>
       </c>
       <c r="F11" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A11,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A11,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G11" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A11,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A11,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H11" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A11,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A11,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I11" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A11,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A11,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J11" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A11,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K11" s="11">
+      <c r="L11" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A11,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A11,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L11" s="11">
+      <c r="M11" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A11,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M11" s="11">
+      <c r="N11" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A11,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N11" s="12">
-        <f>IFERROR(J11/B11,0)</f>
-        <v/>
-      </c>
       <c r="O11" s="12">
+        <f>IFERROR(K11/J11,0)</f>
+        <v/>
+      </c>
+      <c r="P11" s="12">
         <f>IFERROR(I11/B11,0)</f>
         <v/>
       </c>
@@ -1432,7 +1478,7 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A12)</f>
+        <f>C12+D12+E12</f>
         <v/>
       </c>
       <c r="C12" s="11">
@@ -1448,42 +1494,46 @@
         <v/>
       </c>
       <c r="F12" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A12,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A12,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G12" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A12,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A12,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H12" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A12,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A12,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I12" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A12,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A12,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J12" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A12,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K12" s="11">
+      <c r="L12" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A12,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A12,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L12" s="11">
+      <c r="M12" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A12,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M12" s="11">
+      <c r="N12" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A12,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N12" s="12">
-        <f>IFERROR(J12/B12,0)</f>
-        <v/>
-      </c>
       <c r="O12" s="12">
+        <f>IFERROR(K12/J12,0)</f>
+        <v/>
+      </c>
+      <c r="P12" s="12">
         <f>IFERROR(I12/B12,0)</f>
         <v/>
       </c>
@@ -1495,7 +1545,7 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A13)</f>
+        <f>C13+D13+E13</f>
         <v/>
       </c>
       <c r="C13" s="11">
@@ -1511,42 +1561,46 @@
         <v/>
       </c>
       <c r="F13" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A13,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A13,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G13" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A13,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A13,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H13" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A13,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A13,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I13" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A13,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A13,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J13" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A13,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K13" s="11">
+      <c r="L13" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A13,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A13,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L13" s="11">
+      <c r="M13" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A13,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M13" s="11">
+      <c r="N13" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A13,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N13" s="12">
-        <f>IFERROR(J13/B13,0)</f>
-        <v/>
-      </c>
       <c r="O13" s="12">
+        <f>IFERROR(K13/J13,0)</f>
+        <v/>
+      </c>
+      <c r="P13" s="12">
         <f>IFERROR(I13/B13,0)</f>
         <v/>
       </c>
@@ -1558,7 +1612,7 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A14)</f>
+        <f>C14+D14+E14</f>
         <v/>
       </c>
       <c r="C14" s="11">
@@ -1574,42 +1628,46 @@
         <v/>
       </c>
       <c r="F14" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A14,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A14,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G14" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A14,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A14,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H14" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A14,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A14,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I14" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A14,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A14,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J14" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A14,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K14" s="11">
+      <c r="L14" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A14,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A14,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L14" s="11">
+      <c r="M14" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A14,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M14" s="11">
+      <c r="N14" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A14,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N14" s="12">
-        <f>IFERROR(J14/B14,0)</f>
-        <v/>
-      </c>
       <c r="O14" s="12">
+        <f>IFERROR(K14/J14,0)</f>
+        <v/>
+      </c>
+      <c r="P14" s="12">
         <f>IFERROR(I14/B14,0)</f>
         <v/>
       </c>
@@ -1621,7 +1679,7 @@
         </is>
       </c>
       <c r="B15" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A15)</f>
+        <f>C15+D15+E15</f>
         <v/>
       </c>
       <c r="C15" s="11">
@@ -1637,42 +1695,46 @@
         <v/>
       </c>
       <c r="F15" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A15,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A15,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G15" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A15,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A15,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H15" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A15,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A15,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I15" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A15,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A15,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J15" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A15,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K15" s="11">
+      <c r="L15" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A15,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A15,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L15" s="11">
+      <c r="M15" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A15,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M15" s="11">
+      <c r="N15" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A15,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N15" s="12">
-        <f>IFERROR(J15/B15,0)</f>
-        <v/>
-      </c>
       <c r="O15" s="12">
+        <f>IFERROR(K15/J15,0)</f>
+        <v/>
+      </c>
+      <c r="P15" s="12">
         <f>IFERROR(I15/B15,0)</f>
         <v/>
       </c>
@@ -1684,7 +1746,7 @@
         </is>
       </c>
       <c r="B16" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A16)</f>
+        <f>C16+D16+E16</f>
         <v/>
       </c>
       <c r="C16" s="11">
@@ -1700,42 +1762,46 @@
         <v/>
       </c>
       <c r="F16" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A16,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A16,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G16" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A16,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A16,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H16" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A16,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A16,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I16" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A16,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A16,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J16" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A16,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K16" s="11">
+      <c r="L16" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A16,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A16,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L16" s="11">
+      <c r="M16" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A16,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M16" s="11">
+      <c r="N16" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A16,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N16" s="12">
-        <f>IFERROR(J16/B16,0)</f>
-        <v/>
-      </c>
       <c r="O16" s="12">
+        <f>IFERROR(K16/J16,0)</f>
+        <v/>
+      </c>
+      <c r="P16" s="12">
         <f>IFERROR(I16/B16,0)</f>
         <v/>
       </c>
@@ -1747,7 +1813,7 @@
         </is>
       </c>
       <c r="B17" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A17)</f>
+        <f>C17+D17+E17</f>
         <v/>
       </c>
       <c r="C17" s="11">
@@ -1763,42 +1829,46 @@
         <v/>
       </c>
       <c r="F17" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A17,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A17,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G17" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A17,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A17,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H17" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A17,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A17,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I17" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A17,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A17,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J17" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A17,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K17" s="11">
+      <c r="L17" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A17,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A17,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L17" s="11">
+      <c r="M17" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A17,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M17" s="11">
+      <c r="N17" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A17,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N17" s="12">
-        <f>IFERROR(J17/B17,0)</f>
-        <v/>
-      </c>
       <c r="O17" s="12">
+        <f>IFERROR(K17/J17,0)</f>
+        <v/>
+      </c>
+      <c r="P17" s="12">
         <f>IFERROR(I17/B17,0)</f>
         <v/>
       </c>
@@ -1810,7 +1880,7 @@
         </is>
       </c>
       <c r="B18" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A18)</f>
+        <f>C18+D18+E18</f>
         <v/>
       </c>
       <c r="C18" s="11">
@@ -1826,42 +1896,46 @@
         <v/>
       </c>
       <c r="F18" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A18,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A18,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G18" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A18,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A18,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H18" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A18,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A18,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I18" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A18,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A18,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J18" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A18,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K18" s="11">
+      <c r="L18" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A18,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A18,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L18" s="11">
+      <c r="M18" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A18,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M18" s="11">
+      <c r="N18" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A18,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N18" s="12">
-        <f>IFERROR(J18/B18,0)</f>
-        <v/>
-      </c>
       <c r="O18" s="12">
+        <f>IFERROR(K18/J18,0)</f>
+        <v/>
+      </c>
+      <c r="P18" s="12">
         <f>IFERROR(I18/B18,0)</f>
         <v/>
       </c>
@@ -1873,7 +1947,7 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A19)</f>
+        <f>C19+D19+E19</f>
         <v/>
       </c>
       <c r="C19" s="11">
@@ -1889,42 +1963,46 @@
         <v/>
       </c>
       <c r="F19" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A19,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A19,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G19" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A19,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A19,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H19" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A19,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A19,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I19" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A19,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A19,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J19" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A19,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K19" s="11">
+      <c r="L19" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A19,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A19,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L19" s="11">
+      <c r="M19" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A19,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M19" s="11">
+      <c r="N19" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A19,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N19" s="12">
-        <f>IFERROR(J19/B19,0)</f>
-        <v/>
-      </c>
       <c r="O19" s="12">
+        <f>IFERROR(K19/J19,0)</f>
+        <v/>
+      </c>
+      <c r="P19" s="12">
         <f>IFERROR(I19/B19,0)</f>
         <v/>
       </c>
@@ -1936,7 +2014,7 @@
         </is>
       </c>
       <c r="B20" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A20)</f>
+        <f>C20+D20+E20</f>
         <v/>
       </c>
       <c r="C20" s="11">
@@ -1952,42 +2030,46 @@
         <v/>
       </c>
       <c r="F20" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A20,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A20,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G20" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A20,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A20,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H20" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A20,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A20,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I20" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A20,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A20,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J20" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A20,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K20" s="11">
+      <c r="L20" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A20,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A20,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L20" s="11">
+      <c r="M20" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A20,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M20" s="11">
+      <c r="N20" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A20,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N20" s="12">
-        <f>IFERROR(J20/B20,0)</f>
-        <v/>
-      </c>
       <c r="O20" s="12">
+        <f>IFERROR(K20/J20,0)</f>
+        <v/>
+      </c>
+      <c r="P20" s="12">
         <f>IFERROR(I20/B20,0)</f>
         <v/>
       </c>
@@ -1999,7 +2081,7 @@
         </is>
       </c>
       <c r="B21" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A21)</f>
+        <f>C21+D21+E21</f>
         <v/>
       </c>
       <c r="C21" s="11">
@@ -2015,42 +2097,46 @@
         <v/>
       </c>
       <c r="F21" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A21,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A21,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G21" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A21,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A21,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H21" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A21,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A21,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I21" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A21,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A21,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J21" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A21)</f>
+        <v/>
+      </c>
+      <c r="K21" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A21,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K21" s="11">
+      <c r="L21" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A21,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A21,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L21" s="11">
+      <c r="M21" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A21,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M21" s="11">
+      <c r="N21" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A21,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N21" s="12">
-        <f>IFERROR(J21/B21,0)</f>
-        <v/>
-      </c>
       <c r="O21" s="12">
+        <f>IFERROR(K21/J21,0)</f>
+        <v/>
+      </c>
+      <c r="P21" s="12">
         <f>IFERROR(I21/B21,0)</f>
         <v/>
       </c>
@@ -2062,7 +2148,7 @@
         </is>
       </c>
       <c r="B22" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A22)</f>
+        <f>C22+D22+E22</f>
         <v/>
       </c>
       <c r="C22" s="11">
@@ -2078,42 +2164,46 @@
         <v/>
       </c>
       <c r="F22" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A22,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A22,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G22" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A22,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A22,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H22" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A22,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A22,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I22" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A22,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A22,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J22" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A22)</f>
+        <v/>
+      </c>
+      <c r="K22" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A22,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K22" s="11">
+      <c r="L22" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A22,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A22,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L22" s="11">
+      <c r="M22" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A22,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M22" s="11">
+      <c r="N22" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A22,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N22" s="12">
-        <f>IFERROR(J22/B22,0)</f>
-        <v/>
-      </c>
       <c r="O22" s="12">
+        <f>IFERROR(K22/J22,0)</f>
+        <v/>
+      </c>
+      <c r="P22" s="12">
         <f>IFERROR(I22/B22,0)</f>
         <v/>
       </c>
@@ -2125,7 +2215,7 @@
         </is>
       </c>
       <c r="B23" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A23)</f>
+        <f>C23+D23+E23</f>
         <v/>
       </c>
       <c r="C23" s="11">
@@ -2141,42 +2231,46 @@
         <v/>
       </c>
       <c r="F23" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A23,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A23,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G23" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A23,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A23,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H23" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A23,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A23,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I23" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A23,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A23,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J23" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A23)</f>
+        <v/>
+      </c>
+      <c r="K23" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A23,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K23" s="11">
+      <c r="L23" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A23,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A23,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L23" s="11">
+      <c r="M23" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A23,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M23" s="11">
+      <c r="N23" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A23,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N23" s="12">
-        <f>IFERROR(J23/B23,0)</f>
-        <v/>
-      </c>
       <c r="O23" s="12">
+        <f>IFERROR(K23/J23,0)</f>
+        <v/>
+      </c>
+      <c r="P23" s="12">
         <f>IFERROR(I23/B23,0)</f>
         <v/>
       </c>
@@ -2188,7 +2282,7 @@
         </is>
       </c>
       <c r="B24" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A24)</f>
+        <f>C24+D24+E24</f>
         <v/>
       </c>
       <c r="C24" s="11">
@@ -2204,42 +2298,46 @@
         <v/>
       </c>
       <c r="F24" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A24,RTM!$H$2:$H$335,"M")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A24,RTM!$H$2:$H$335,"M",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="G24" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A24,RTM!$H$2:$H$335,"S")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A24,RTM!$H$2:$H$335,"S",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="H24" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A24,RTM!$H$2:$H$335,"C")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A24,RTM!$H$2:$H$335,"C",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="I24" s="11">
-        <f>COUNTIFS(RTM!$C$2:$C$335,$A24,RTM!$I$2:$I$335,"?*")</f>
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A24,RTM!$I$2:$I$335,"?*",RTM!$B$2:$B$335,"&lt;&gt;Additional Test Case")</f>
         <v/>
       </c>
       <c r="J24" s="11">
+        <f>COUNTIFS(RTM!$C$2:$C$335,$A24)</f>
+        <v/>
+      </c>
+      <c r="K24" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A24,RTM!$N$2:$N$335,"Passed")</f>
         <v/>
       </c>
-      <c r="K24" s="11">
+      <c r="L24" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A24,RTM!$N$2:$N$335,"Failed")+COUNTIFS(RTM!$C$2:$C$335,$A24,RTM!$N$2:$N$335,"Blocked")</f>
         <v/>
       </c>
-      <c r="L24" s="11">
+      <c r="M24" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A24,RTM!$N$2:$N$335,"In Progress")</f>
         <v/>
       </c>
-      <c r="M24" s="11">
+      <c r="N24" s="11">
         <f>COUNTIFS(RTM!$C$2:$C$335,$A24,RTM!$N$2:$N$335,"Not Started")</f>
         <v/>
       </c>
-      <c r="N24" s="12">
-        <f>IFERROR(J24/B24,0)</f>
-        <v/>
-      </c>
       <c r="O24" s="12">
+        <f>IFERROR(K24/J24,0)</f>
+        <v/>
+      </c>
+      <c r="P24" s="12">
         <f>IFERROR(I24/B24,0)</f>
         <v/>
       </c>
@@ -2298,11 +2396,15 @@
         <f>SUM(M5:M24)</f>
         <v/>
       </c>
-      <c r="N25" s="15">
-        <f>IFERROR(J25/B25,0)</f>
+      <c r="N25" s="14">
+        <f>SUM(N5:N24)</f>
         <v/>
       </c>
       <c r="O25" s="15">
+        <f>IFERROR(K25/J25,0)</f>
+        <v/>
+      </c>
+      <c r="P25" s="15">
         <f>IFERROR(I25/B25,0)</f>
         <v/>
       </c>
@@ -2318,7 +2420,7 @@
         <v/>
       </c>
       <c r="C27" s="16">
-        <f>IF(B27=B25,"OK - all rows mapped to an area","MISMATCH")</f>
+        <f>IF(B27=J25,"OK - all rows mapped to an area","MISMATCH")</f>
         <v/>
       </c>
     </row>
@@ -2507,7 +2609,7 @@
       </c>
       <c r="O2" s="18" t="n"/>
       <c r="P2" s="18" t="n"/>
-      <c r="Q2" s="18" t="inlineStr"/>
+      <c r="Q2" s="18" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
@@ -2574,7 +2676,7 @@
       </c>
       <c r="O3" s="18" t="n"/>
       <c r="P3" s="18" t="n"/>
-      <c r="Q3" s="18" t="inlineStr"/>
+      <c r="Q3" s="18" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="18" t="inlineStr">
@@ -2641,7 +2743,7 @@
       </c>
       <c r="O4" s="18" t="n"/>
       <c r="P4" s="18" t="n"/>
-      <c r="Q4" s="18" t="inlineStr"/>
+      <c r="Q4" s="18" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="18" t="inlineStr">
@@ -2708,7 +2810,7 @@
       </c>
       <c r="O5" s="18" t="n"/>
       <c r="P5" s="18" t="n"/>
-      <c r="Q5" s="18" t="inlineStr"/>
+      <c r="Q5" s="18" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="18" t="inlineStr">
@@ -2775,7 +2877,7 @@
       </c>
       <c r="O6" s="18" t="n"/>
       <c r="P6" s="18" t="n"/>
-      <c r="Q6" s="18" t="inlineStr"/>
+      <c r="Q6" s="18" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
@@ -2842,7 +2944,7 @@
       </c>
       <c r="O7" s="18" t="n"/>
       <c r="P7" s="18" t="n"/>
-      <c r="Q7" s="18" t="inlineStr"/>
+      <c r="Q7" s="18" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="18" t="inlineStr">
@@ -2909,7 +3011,7 @@
       </c>
       <c r="O8" s="18" t="n"/>
       <c r="P8" s="18" t="n"/>
-      <c r="Q8" s="18" t="inlineStr"/>
+      <c r="Q8" s="18" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="18" t="inlineStr">
@@ -2976,7 +3078,7 @@
       </c>
       <c r="O9" s="18" t="n"/>
       <c r="P9" s="18" t="n"/>
-      <c r="Q9" s="18" t="inlineStr"/>
+      <c r="Q9" s="18" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="18" t="inlineStr">
@@ -3043,7 +3145,7 @@
       </c>
       <c r="O10" s="18" t="n"/>
       <c r="P10" s="18" t="n"/>
-      <c r="Q10" s="18" t="inlineStr"/>
+      <c r="Q10" s="18" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
@@ -3110,7 +3212,7 @@
       </c>
       <c r="O11" s="18" t="n"/>
       <c r="P11" s="18" t="n"/>
-      <c r="Q11" s="18" t="inlineStr"/>
+      <c r="Q11" s="18" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
@@ -3177,7 +3279,7 @@
       </c>
       <c r="O12" s="18" t="n"/>
       <c r="P12" s="18" t="n"/>
-      <c r="Q12" s="18" t="inlineStr"/>
+      <c r="Q12" s="18" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="18" t="inlineStr">
@@ -3244,7 +3346,7 @@
       </c>
       <c r="O13" s="18" t="n"/>
       <c r="P13" s="18" t="n"/>
-      <c r="Q13" s="18" t="inlineStr"/>
+      <c r="Q13" s="18" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
@@ -4092,7 +4194,7 @@
       </c>
       <c r="O25" s="18" t="n"/>
       <c r="P25" s="18" t="n"/>
-      <c r="Q25" s="18" t="inlineStr"/>
+      <c r="Q25" s="18" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="18" t="inlineStr">
@@ -4159,7 +4261,7 @@
       </c>
       <c r="O26" s="18" t="n"/>
       <c r="P26" s="18" t="n"/>
-      <c r="Q26" s="18" t="inlineStr"/>
+      <c r="Q26" s="18" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="18" t="inlineStr">
@@ -4226,7 +4328,7 @@
       </c>
       <c r="O27" s="18" t="n"/>
       <c r="P27" s="18" t="n"/>
-      <c r="Q27" s="18" t="inlineStr"/>
+      <c r="Q27" s="18" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
@@ -4293,7 +4395,7 @@
       </c>
       <c r="O28" s="18" t="n"/>
       <c r="P28" s="18" t="n"/>
-      <c r="Q28" s="18" t="inlineStr"/>
+      <c r="Q28" s="18" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="18" t="inlineStr">
@@ -4360,7 +4462,7 @@
       </c>
       <c r="O29" s="18" t="n"/>
       <c r="P29" s="18" t="n"/>
-      <c r="Q29" s="18" t="inlineStr"/>
+      <c r="Q29" s="18" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="18" t="inlineStr">
@@ -4427,7 +4529,7 @@
       </c>
       <c r="O30" s="18" t="n"/>
       <c r="P30" s="18" t="n"/>
-      <c r="Q30" s="18" t="inlineStr"/>
+      <c r="Q30" s="18" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="18" t="inlineStr">
@@ -4494,7 +4596,7 @@
       </c>
       <c r="O31" s="18" t="n"/>
       <c r="P31" s="18" t="n"/>
-      <c r="Q31" s="18" t="inlineStr"/>
+      <c r="Q31" s="18" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="18" t="inlineStr">
@@ -4561,7 +4663,7 @@
       </c>
       <c r="O32" s="18" t="n"/>
       <c r="P32" s="18" t="n"/>
-      <c r="Q32" s="18" t="inlineStr"/>
+      <c r="Q32" s="18" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="18" t="inlineStr">
@@ -5054,7 +5156,7 @@
       </c>
       <c r="O39" s="18" t="n"/>
       <c r="P39" s="18" t="n"/>
-      <c r="Q39" s="18" t="inlineStr"/>
+      <c r="Q39" s="18" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="18" t="inlineStr">
@@ -5121,7 +5223,7 @@
       </c>
       <c r="O40" s="18" t="n"/>
       <c r="P40" s="18" t="n"/>
-      <c r="Q40" s="18" t="inlineStr"/>
+      <c r="Q40" s="18" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="18" t="inlineStr">
@@ -5188,7 +5290,7 @@
       </c>
       <c r="O41" s="18" t="n"/>
       <c r="P41" s="18" t="n"/>
-      <c r="Q41" s="18" t="inlineStr"/>
+      <c r="Q41" s="18" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="18" t="inlineStr">
@@ -5255,7 +5357,7 @@
       </c>
       <c r="O42" s="18" t="n"/>
       <c r="P42" s="18" t="n"/>
-      <c r="Q42" s="18" t="inlineStr"/>
+      <c r="Q42" s="18" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="18" t="inlineStr">
@@ -5322,7 +5424,7 @@
       </c>
       <c r="O43" s="18" t="n"/>
       <c r="P43" s="18" t="n"/>
-      <c r="Q43" s="18" t="inlineStr"/>
+      <c r="Q43" s="18" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="18" t="inlineStr">
@@ -5389,7 +5491,7 @@
       </c>
       <c r="O44" s="18" t="n"/>
       <c r="P44" s="18" t="n"/>
-      <c r="Q44" s="18" t="inlineStr"/>
+      <c r="Q44" s="18" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="18" t="inlineStr">
@@ -5811,7 +5913,7 @@
       </c>
       <c r="O50" s="18" t="n"/>
       <c r="P50" s="18" t="n"/>
-      <c r="Q50" s="18" t="inlineStr"/>
+      <c r="Q50" s="18" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="18" t="inlineStr">
@@ -5878,7 +5980,7 @@
       </c>
       <c r="O51" s="18" t="n"/>
       <c r="P51" s="18" t="n"/>
-      <c r="Q51" s="18" t="inlineStr"/>
+      <c r="Q51" s="18" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="18" t="inlineStr">
@@ -5945,7 +6047,7 @@
       </c>
       <c r="O52" s="18" t="n"/>
       <c r="P52" s="18" t="n"/>
-      <c r="Q52" s="18" t="inlineStr"/>
+      <c r="Q52" s="18" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="18" t="inlineStr">
@@ -6012,7 +6114,7 @@
       </c>
       <c r="O53" s="18" t="n"/>
       <c r="P53" s="18" t="n"/>
-      <c r="Q53" s="18" t="inlineStr"/>
+      <c r="Q53" s="18" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="18" t="inlineStr">
@@ -6079,7 +6181,7 @@
       </c>
       <c r="O54" s="18" t="n"/>
       <c r="P54" s="18" t="n"/>
-      <c r="Q54" s="18" t="inlineStr"/>
+      <c r="Q54" s="18" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="18" t="inlineStr">
@@ -6146,7 +6248,7 @@
       </c>
       <c r="O55" s="18" t="n"/>
       <c r="P55" s="18" t="n"/>
-      <c r="Q55" s="18" t="inlineStr"/>
+      <c r="Q55" s="18" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="18" t="inlineStr">
@@ -6213,7 +6315,7 @@
       </c>
       <c r="O56" s="18" t="n"/>
       <c r="P56" s="18" t="n"/>
-      <c r="Q56" s="18" t="inlineStr"/>
+      <c r="Q56" s="18" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="18" t="inlineStr">
@@ -6280,7 +6382,7 @@
       </c>
       <c r="O57" s="18" t="n"/>
       <c r="P57" s="18" t="n"/>
-      <c r="Q57" s="18" t="inlineStr"/>
+      <c r="Q57" s="18" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="18" t="inlineStr">
@@ -6347,7 +6449,7 @@
       </c>
       <c r="O58" s="18" t="n"/>
       <c r="P58" s="18" t="n"/>
-      <c r="Q58" s="18" t="inlineStr"/>
+      <c r="Q58" s="18" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="18" t="inlineStr">
@@ -6911,7 +7013,7 @@
       </c>
       <c r="O66" s="18" t="n"/>
       <c r="P66" s="18" t="n"/>
-      <c r="Q66" s="18" t="inlineStr"/>
+      <c r="Q66" s="18" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="18" t="inlineStr">
@@ -6978,7 +7080,7 @@
       </c>
       <c r="O67" s="18" t="n"/>
       <c r="P67" s="18" t="n"/>
-      <c r="Q67" s="18" t="inlineStr"/>
+      <c r="Q67" s="18" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="18" t="inlineStr">
@@ -7045,7 +7147,7 @@
       </c>
       <c r="O68" s="18" t="n"/>
       <c r="P68" s="18" t="n"/>
-      <c r="Q68" s="18" t="inlineStr"/>
+      <c r="Q68" s="18" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="18" t="inlineStr">
@@ -7112,7 +7214,7 @@
       </c>
       <c r="O69" s="18" t="n"/>
       <c r="P69" s="18" t="n"/>
-      <c r="Q69" s="18" t="inlineStr"/>
+      <c r="Q69" s="18" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
@@ -7179,7 +7281,7 @@
       </c>
       <c r="O70" s="18" t="n"/>
       <c r="P70" s="18" t="n"/>
-      <c r="Q70" s="18" t="inlineStr"/>
+      <c r="Q70" s="18" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="18" t="inlineStr">
@@ -7246,7 +7348,7 @@
       </c>
       <c r="O71" s="18" t="n"/>
       <c r="P71" s="18" t="n"/>
-      <c r="Q71" s="18" t="inlineStr"/>
+      <c r="Q71" s="18" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="18" t="inlineStr">
@@ -7313,7 +7415,7 @@
       </c>
       <c r="O72" s="18" t="n"/>
       <c r="P72" s="18" t="n"/>
-      <c r="Q72" s="18" t="inlineStr"/>
+      <c r="Q72" s="18" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
@@ -7806,7 +7908,7 @@
       </c>
       <c r="O79" s="18" t="n"/>
       <c r="P79" s="18" t="n"/>
-      <c r="Q79" s="18" t="inlineStr"/>
+      <c r="Q79" s="18" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
@@ -7873,7 +7975,7 @@
       </c>
       <c r="O80" s="18" t="n"/>
       <c r="P80" s="18" t="n"/>
-      <c r="Q80" s="18" t="inlineStr"/>
+      <c r="Q80" s="18" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="18" t="inlineStr">
@@ -7940,7 +8042,7 @@
       </c>
       <c r="O81" s="18" t="n"/>
       <c r="P81" s="18" t="n"/>
-      <c r="Q81" s="18" t="inlineStr"/>
+      <c r="Q81" s="18" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="18" t="inlineStr">
@@ -8007,7 +8109,7 @@
       </c>
       <c r="O82" s="18" t="n"/>
       <c r="P82" s="18" t="n"/>
-      <c r="Q82" s="18" t="inlineStr"/>
+      <c r="Q82" s="18" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="18" t="inlineStr">
@@ -8074,7 +8176,7 @@
       </c>
       <c r="O83" s="18" t="n"/>
       <c r="P83" s="18" t="n"/>
-      <c r="Q83" s="18" t="inlineStr"/>
+      <c r="Q83" s="18" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="18" t="inlineStr">
@@ -8141,7 +8243,7 @@
       </c>
       <c r="O84" s="18" t="n"/>
       <c r="P84" s="18" t="n"/>
-      <c r="Q84" s="18" t="inlineStr"/>
+      <c r="Q84" s="18" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="18" t="inlineStr">
@@ -8208,7 +8310,7 @@
       </c>
       <c r="O85" s="18" t="n"/>
       <c r="P85" s="18" t="n"/>
-      <c r="Q85" s="18" t="inlineStr"/>
+      <c r="Q85" s="18" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="18" t="inlineStr">
@@ -8275,7 +8377,7 @@
       </c>
       <c r="O86" s="18" t="n"/>
       <c r="P86" s="18" t="n"/>
-      <c r="Q86" s="18" t="inlineStr"/>
+      <c r="Q86" s="18" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
@@ -8626,7 +8728,7 @@
       </c>
       <c r="O91" s="18" t="n"/>
       <c r="P91" s="18" t="n"/>
-      <c r="Q91" s="18" t="inlineStr"/>
+      <c r="Q91" s="18" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
@@ -8693,7 +8795,7 @@
       </c>
       <c r="O92" s="18" t="n"/>
       <c r="P92" s="18" t="n"/>
-      <c r="Q92" s="18" t="inlineStr"/>
+      <c r="Q92" s="18" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="18" t="inlineStr">
@@ -8760,7 +8862,7 @@
       </c>
       <c r="O93" s="18" t="n"/>
       <c r="P93" s="18" t="n"/>
-      <c r="Q93" s="18" t="inlineStr"/>
+      <c r="Q93" s="18" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
@@ -8827,7 +8929,7 @@
       </c>
       <c r="O94" s="18" t="n"/>
       <c r="P94" s="18" t="n"/>
-      <c r="Q94" s="18" t="inlineStr"/>
+      <c r="Q94" s="18" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="18" t="inlineStr">
@@ -8894,7 +8996,7 @@
       </c>
       <c r="O95" s="18" t="n"/>
       <c r="P95" s="18" t="n"/>
-      <c r="Q95" s="18" t="inlineStr"/>
+      <c r="Q95" s="18" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="18" t="inlineStr">
@@ -9174,7 +9276,7 @@
       </c>
       <c r="O99" s="18" t="n"/>
       <c r="P99" s="18" t="n"/>
-      <c r="Q99" s="18" t="inlineStr"/>
+      <c r="Q99" s="18" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="18" t="inlineStr">
@@ -9241,7 +9343,7 @@
       </c>
       <c r="O100" s="18" t="n"/>
       <c r="P100" s="18" t="n"/>
-      <c r="Q100" s="18" t="inlineStr"/>
+      <c r="Q100" s="18" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="18" t="inlineStr">
@@ -9308,7 +9410,7 @@
       </c>
       <c r="O101" s="18" t="n"/>
       <c r="P101" s="18" t="n"/>
-      <c r="Q101" s="18" t="inlineStr"/>
+      <c r="Q101" s="18" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="18" t="inlineStr">
@@ -9375,7 +9477,7 @@
       </c>
       <c r="O102" s="18" t="n"/>
       <c r="P102" s="18" t="n"/>
-      <c r="Q102" s="18" t="inlineStr"/>
+      <c r="Q102" s="18" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="18" t="inlineStr">
@@ -9442,7 +9544,7 @@
       </c>
       <c r="O103" s="18" t="n"/>
       <c r="P103" s="18" t="n"/>
-      <c r="Q103" s="18" t="inlineStr"/>
+      <c r="Q103" s="18" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="18" t="inlineStr">
@@ -9509,7 +9611,7 @@
       </c>
       <c r="O104" s="18" t="n"/>
       <c r="P104" s="18" t="n"/>
-      <c r="Q104" s="18" t="inlineStr"/>
+      <c r="Q104" s="18" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="18" t="inlineStr">
@@ -9860,7 +9962,7 @@
       </c>
       <c r="O109" s="18" t="n"/>
       <c r="P109" s="18" t="n"/>
-      <c r="Q109" s="18" t="inlineStr"/>
+      <c r="Q109" s="18" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="18" t="inlineStr">
@@ -9927,7 +10029,7 @@
       </c>
       <c r="O110" s="18" t="n"/>
       <c r="P110" s="18" t="n"/>
-      <c r="Q110" s="18" t="inlineStr"/>
+      <c r="Q110" s="18" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="18" t="inlineStr">
@@ -9994,7 +10096,7 @@
       </c>
       <c r="O111" s="18" t="n"/>
       <c r="P111" s="18" t="n"/>
-      <c r="Q111" s="18" t="inlineStr"/>
+      <c r="Q111" s="18" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="18" t="inlineStr">
@@ -10061,7 +10163,7 @@
       </c>
       <c r="O112" s="18" t="n"/>
       <c r="P112" s="18" t="n"/>
-      <c r="Q112" s="18" t="inlineStr"/>
+      <c r="Q112" s="18" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="18" t="inlineStr">
@@ -10341,7 +10443,7 @@
       </c>
       <c r="O116" s="18" t="n"/>
       <c r="P116" s="18" t="n"/>
-      <c r="Q116" s="18" t="inlineStr"/>
+      <c r="Q116" s="18" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="18" t="inlineStr">
@@ -10408,7 +10510,7 @@
       </c>
       <c r="O117" s="18" t="n"/>
       <c r="P117" s="18" t="n"/>
-      <c r="Q117" s="18" t="inlineStr"/>
+      <c r="Q117" s="18" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="18" t="inlineStr">
@@ -10475,7 +10577,7 @@
       </c>
       <c r="O118" s="18" t="n"/>
       <c r="P118" s="18" t="n"/>
-      <c r="Q118" s="18" t="inlineStr"/>
+      <c r="Q118" s="18" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="18" t="inlineStr">
@@ -10542,7 +10644,7 @@
       </c>
       <c r="O119" s="18" t="n"/>
       <c r="P119" s="18" t="n"/>
-      <c r="Q119" s="18" t="inlineStr"/>
+      <c r="Q119" s="18" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="18" t="inlineStr">
@@ -10822,7 +10924,7 @@
       </c>
       <c r="O123" s="18" t="n"/>
       <c r="P123" s="18" t="n"/>
-      <c r="Q123" s="18" t="inlineStr"/>
+      <c r="Q123" s="18" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="18" t="inlineStr">
@@ -10889,7 +10991,7 @@
       </c>
       <c r="O124" s="18" t="n"/>
       <c r="P124" s="18" t="n"/>
-      <c r="Q124" s="18" t="inlineStr"/>
+      <c r="Q124" s="18" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="18" t="inlineStr">
@@ -10956,7 +11058,7 @@
       </c>
       <c r="O125" s="18" t="n"/>
       <c r="P125" s="18" t="n"/>
-      <c r="Q125" s="18" t="inlineStr"/>
+      <c r="Q125" s="18" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="18" t="inlineStr">
@@ -11023,7 +11125,7 @@
       </c>
       <c r="O126" s="18" t="n"/>
       <c r="P126" s="18" t="n"/>
-      <c r="Q126" s="18" t="inlineStr"/>
+      <c r="Q126" s="18" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="18" t="inlineStr">
@@ -11090,7 +11192,7 @@
       </c>
       <c r="O127" s="18" t="n"/>
       <c r="P127" s="18" t="n"/>
-      <c r="Q127" s="18" t="inlineStr"/>
+      <c r="Q127" s="18" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="18" t="inlineStr">
@@ -11370,7 +11472,7 @@
       </c>
       <c r="O131" s="18" t="n"/>
       <c r="P131" s="18" t="n"/>
-      <c r="Q131" s="18" t="inlineStr"/>
+      <c r="Q131" s="18" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="18" t="inlineStr">
@@ -11437,7 +11539,7 @@
       </c>
       <c r="O132" s="18" t="n"/>
       <c r="P132" s="18" t="n"/>
-      <c r="Q132" s="18" t="inlineStr"/>
+      <c r="Q132" s="18" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="18" t="inlineStr">
@@ -11504,7 +11606,7 @@
       </c>
       <c r="O133" s="18" t="n"/>
       <c r="P133" s="18" t="n"/>
-      <c r="Q133" s="18" t="inlineStr"/>
+      <c r="Q133" s="18" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="18" t="inlineStr">
@@ -11571,7 +11673,7 @@
       </c>
       <c r="O134" s="18" t="n"/>
       <c r="P134" s="18" t="n"/>
-      <c r="Q134" s="18" t="inlineStr"/>
+      <c r="Q134" s="18" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="18" t="inlineStr">
@@ -11638,7 +11740,7 @@
       </c>
       <c r="O135" s="18" t="n"/>
       <c r="P135" s="18" t="n"/>
-      <c r="Q135" s="18" t="inlineStr"/>
+      <c r="Q135" s="18" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="18" t="inlineStr">
@@ -11918,7 +12020,7 @@
       </c>
       <c r="O139" s="18" t="n"/>
       <c r="P139" s="18" t="n"/>
-      <c r="Q139" s="18" t="inlineStr"/>
+      <c r="Q139" s="18" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="18" t="inlineStr">
@@ -11985,7 +12087,7 @@
       </c>
       <c r="O140" s="18" t="n"/>
       <c r="P140" s="18" t="n"/>
-      <c r="Q140" s="18" t="inlineStr"/>
+      <c r="Q140" s="18" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="18" t="inlineStr">
@@ -12052,7 +12154,7 @@
       </c>
       <c r="O141" s="18" t="n"/>
       <c r="P141" s="18" t="n"/>
-      <c r="Q141" s="18" t="inlineStr"/>
+      <c r="Q141" s="18" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="18" t="inlineStr">
@@ -12119,7 +12221,7 @@
       </c>
       <c r="O142" s="18" t="n"/>
       <c r="P142" s="18" t="n"/>
-      <c r="Q142" s="18" t="inlineStr"/>
+      <c r="Q142" s="18" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="18" t="inlineStr">
@@ -12186,7 +12288,7 @@
       </c>
       <c r="O143" s="18" t="n"/>
       <c r="P143" s="18" t="n"/>
-      <c r="Q143" s="18" t="inlineStr"/>
+      <c r="Q143" s="18" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="18" t="inlineStr">
@@ -12466,7 +12568,7 @@
       </c>
       <c r="O147" s="18" t="n"/>
       <c r="P147" s="18" t="n"/>
-      <c r="Q147" s="18" t="inlineStr"/>
+      <c r="Q147" s="18" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="18" t="inlineStr">
@@ -12533,7 +12635,7 @@
       </c>
       <c r="O148" s="18" t="n"/>
       <c r="P148" s="18" t="n"/>
-      <c r="Q148" s="18" t="inlineStr"/>
+      <c r="Q148" s="18" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="18" t="inlineStr">
@@ -12600,7 +12702,7 @@
       </c>
       <c r="O149" s="18" t="n"/>
       <c r="P149" s="18" t="n"/>
-      <c r="Q149" s="18" t="inlineStr"/>
+      <c r="Q149" s="18" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="18" t="inlineStr">
@@ -12667,7 +12769,7 @@
       </c>
       <c r="O150" s="18" t="n"/>
       <c r="P150" s="18" t="n"/>
-      <c r="Q150" s="18" t="inlineStr"/>
+      <c r="Q150" s="18" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="18" t="inlineStr">
@@ -12734,7 +12836,7 @@
       </c>
       <c r="O151" s="18" t="n"/>
       <c r="P151" s="18" t="n"/>
-      <c r="Q151" s="18" t="inlineStr"/>
+      <c r="Q151" s="18" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="18" t="inlineStr">
@@ -12801,7 +12903,7 @@
       </c>
       <c r="O152" s="18" t="n"/>
       <c r="P152" s="18" t="n"/>
-      <c r="Q152" s="18" t="inlineStr"/>
+      <c r="Q152" s="18" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="18" t="inlineStr">
@@ -13223,7 +13325,7 @@
       </c>
       <c r="O158" s="18" t="n"/>
       <c r="P158" s="18" t="n"/>
-      <c r="Q158" s="18" t="inlineStr"/>
+      <c r="Q158" s="18" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="18" t="inlineStr">
@@ -13290,7 +13392,7 @@
       </c>
       <c r="O159" s="18" t="n"/>
       <c r="P159" s="18" t="n"/>
-      <c r="Q159" s="18" t="inlineStr"/>
+      <c r="Q159" s="18" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="18" t="inlineStr">
@@ -13357,7 +13459,7 @@
       </c>
       <c r="O160" s="18" t="n"/>
       <c r="P160" s="18" t="n"/>
-      <c r="Q160" s="18" t="inlineStr"/>
+      <c r="Q160" s="18" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="18" t="inlineStr">
@@ -13424,7 +13526,7 @@
       </c>
       <c r="O161" s="18" t="n"/>
       <c r="P161" s="18" t="n"/>
-      <c r="Q161" s="18" t="inlineStr"/>
+      <c r="Q161" s="18" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="18" t="inlineStr">
@@ -13491,7 +13593,7 @@
       </c>
       <c r="O162" s="18" t="n"/>
       <c r="P162" s="18" t="n"/>
-      <c r="Q162" s="18" t="inlineStr"/>
+      <c r="Q162" s="18" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="18" t="inlineStr">
@@ -13558,7 +13660,7 @@
       </c>
       <c r="O163" s="18" t="n"/>
       <c r="P163" s="18" t="n"/>
-      <c r="Q163" s="18" t="inlineStr"/>
+      <c r="Q163" s="18" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="18" t="inlineStr">
@@ -13625,7 +13727,7 @@
       </c>
       <c r="O164" s="18" t="n"/>
       <c r="P164" s="18" t="n"/>
-      <c r="Q164" s="18" t="inlineStr"/>
+      <c r="Q164" s="18" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="18" t="inlineStr">
@@ -13692,7 +13794,7 @@
       </c>
       <c r="O165" s="18" t="n"/>
       <c r="P165" s="18" t="n"/>
-      <c r="Q165" s="18" t="inlineStr"/>
+      <c r="Q165" s="18" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="18" t="inlineStr">
@@ -13759,7 +13861,7 @@
       </c>
       <c r="O166" s="18" t="n"/>
       <c r="P166" s="18" t="n"/>
-      <c r="Q166" s="18" t="inlineStr"/>
+      <c r="Q166" s="18" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="18" t="inlineStr">
@@ -13826,7 +13928,7 @@
       </c>
       <c r="O167" s="18" t="n"/>
       <c r="P167" s="18" t="n"/>
-      <c r="Q167" s="18" t="inlineStr"/>
+      <c r="Q167" s="18" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="18" t="inlineStr">
@@ -13893,7 +13995,7 @@
       </c>
       <c r="O168" s="18" t="n"/>
       <c r="P168" s="18" t="n"/>
-      <c r="Q168" s="18" t="inlineStr"/>
+      <c r="Q168" s="18" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="18" t="inlineStr">
@@ -13960,7 +14062,7 @@
       </c>
       <c r="O169" s="18" t="n"/>
       <c r="P169" s="18" t="n"/>
-      <c r="Q169" s="18" t="inlineStr"/>
+      <c r="Q169" s="18" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="18" t="inlineStr">
@@ -14027,7 +14129,7 @@
       </c>
       <c r="O170" s="18" t="n"/>
       <c r="P170" s="18" t="n"/>
-      <c r="Q170" s="18" t="inlineStr"/>
+      <c r="Q170" s="18" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="18" t="inlineStr">
@@ -14094,7 +14196,7 @@
       </c>
       <c r="O171" s="18" t="n"/>
       <c r="P171" s="18" t="n"/>
-      <c r="Q171" s="18" t="inlineStr"/>
+      <c r="Q171" s="18" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="18" t="inlineStr">
@@ -14161,7 +14263,7 @@
       </c>
       <c r="O172" s="18" t="n"/>
       <c r="P172" s="18" t="n"/>
-      <c r="Q172" s="18" t="inlineStr"/>
+      <c r="Q172" s="18" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="18" t="inlineStr">
@@ -14228,7 +14330,7 @@
       </c>
       <c r="O173" s="18" t="n"/>
       <c r="P173" s="18" t="n"/>
-      <c r="Q173" s="18" t="inlineStr"/>
+      <c r="Q173" s="18" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="18" t="inlineStr">
@@ -14295,7 +14397,7 @@
       </c>
       <c r="O174" s="18" t="n"/>
       <c r="P174" s="18" t="n"/>
-      <c r="Q174" s="18" t="inlineStr"/>
+      <c r="Q174" s="18" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="18" t="inlineStr">
@@ -14433,7 +14535,7 @@
       </c>
       <c r="O176" s="18" t="n"/>
       <c r="P176" s="18" t="n"/>
-      <c r="Q176" s="18" t="inlineStr"/>
+      <c r="Q176" s="18" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="18" t="inlineStr">
@@ -14500,7 +14602,7 @@
       </c>
       <c r="O177" s="18" t="n"/>
       <c r="P177" s="18" t="n"/>
-      <c r="Q177" s="18" t="inlineStr"/>
+      <c r="Q177" s="18" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="18" t="inlineStr">
@@ -14567,7 +14669,7 @@
       </c>
       <c r="O178" s="18" t="n"/>
       <c r="P178" s="18" t="n"/>
-      <c r="Q178" s="18" t="inlineStr"/>
+      <c r="Q178" s="18" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="18" t="inlineStr">
@@ -14634,7 +14736,7 @@
       </c>
       <c r="O179" s="18" t="n"/>
       <c r="P179" s="18" t="n"/>
-      <c r="Q179" s="18" t="inlineStr"/>
+      <c r="Q179" s="18" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="18" t="inlineStr">
@@ -14701,7 +14803,7 @@
       </c>
       <c r="O180" s="18" t="n"/>
       <c r="P180" s="18" t="n"/>
-      <c r="Q180" s="18" t="inlineStr"/>
+      <c r="Q180" s="18" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="18" t="inlineStr">
@@ -14768,7 +14870,7 @@
       </c>
       <c r="O181" s="18" t="n"/>
       <c r="P181" s="18" t="n"/>
-      <c r="Q181" s="18" t="inlineStr"/>
+      <c r="Q181" s="18" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="18" t="inlineStr">
@@ -14835,7 +14937,7 @@
       </c>
       <c r="O182" s="18" t="n"/>
       <c r="P182" s="18" t="n"/>
-      <c r="Q182" s="18" t="inlineStr"/>
+      <c r="Q182" s="18" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="18" t="inlineStr">
@@ -14902,7 +15004,7 @@
       </c>
       <c r="O183" s="18" t="n"/>
       <c r="P183" s="18" t="n"/>
-      <c r="Q183" s="18" t="inlineStr"/>
+      <c r="Q183" s="18" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="18" t="inlineStr">
@@ -14969,7 +15071,7 @@
       </c>
       <c r="O184" s="18" t="n"/>
       <c r="P184" s="18" t="n"/>
-      <c r="Q184" s="18" t="inlineStr"/>
+      <c r="Q184" s="18" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="18" t="inlineStr">
@@ -15036,7 +15138,7 @@
       </c>
       <c r="O185" s="18" t="n"/>
       <c r="P185" s="18" t="n"/>
-      <c r="Q185" s="18" t="inlineStr"/>
+      <c r="Q185" s="18" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="18" t="inlineStr">
@@ -15103,7 +15205,7 @@
       </c>
       <c r="O186" s="18" t="n"/>
       <c r="P186" s="18" t="n"/>
-      <c r="Q186" s="18" t="inlineStr"/>
+      <c r="Q186" s="18" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="18" t="inlineStr">
@@ -15241,7 +15343,7 @@
       </c>
       <c r="O188" s="18" t="n"/>
       <c r="P188" s="18" t="n"/>
-      <c r="Q188" s="18" t="inlineStr"/>
+      <c r="Q188" s="18" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="18" t="inlineStr">
@@ -15308,7 +15410,7 @@
       </c>
       <c r="O189" s="18" t="n"/>
       <c r="P189" s="18" t="n"/>
-      <c r="Q189" s="18" t="inlineStr"/>
+      <c r="Q189" s="18" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="18" t="inlineStr">
@@ -15375,7 +15477,7 @@
       </c>
       <c r="O190" s="18" t="n"/>
       <c r="P190" s="18" t="n"/>
-      <c r="Q190" s="18" t="inlineStr"/>
+      <c r="Q190" s="18" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="18" t="inlineStr">
@@ -15442,7 +15544,7 @@
       </c>
       <c r="O191" s="18" t="n"/>
       <c r="P191" s="18" t="n"/>
-      <c r="Q191" s="18" t="inlineStr"/>
+      <c r="Q191" s="18" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="18" t="inlineStr">
@@ -15509,7 +15611,7 @@
       </c>
       <c r="O192" s="18" t="n"/>
       <c r="P192" s="18" t="n"/>
-      <c r="Q192" s="18" t="inlineStr"/>
+      <c r="Q192" s="18" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="18" t="inlineStr">
@@ -15576,7 +15678,7 @@
       </c>
       <c r="O193" s="18" t="n"/>
       <c r="P193" s="18" t="n"/>
-      <c r="Q193" s="18" t="inlineStr"/>
+      <c r="Q193" s="18" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="18" t="inlineStr">
@@ -15643,7 +15745,7 @@
       </c>
       <c r="O194" s="18" t="n"/>
       <c r="P194" s="18" t="n"/>
-      <c r="Q194" s="18" t="inlineStr"/>
+      <c r="Q194" s="18" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="18" t="inlineStr">
@@ -15710,7 +15812,7 @@
       </c>
       <c r="O195" s="18" t="n"/>
       <c r="P195" s="18" t="n"/>
-      <c r="Q195" s="18" t="inlineStr"/>
+      <c r="Q195" s="18" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="18" t="inlineStr">
@@ -15777,7 +15879,7 @@
       </c>
       <c r="O196" s="18" t="n"/>
       <c r="P196" s="18" t="n"/>
-      <c r="Q196" s="18" t="inlineStr"/>
+      <c r="Q196" s="18" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="18" t="inlineStr">
@@ -15844,7 +15946,7 @@
       </c>
       <c r="O197" s="18" t="n"/>
       <c r="P197" s="18" t="n"/>
-      <c r="Q197" s="18" t="inlineStr"/>
+      <c r="Q197" s="18" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="18" t="inlineStr">
@@ -15911,7 +16013,7 @@
       </c>
       <c r="O198" s="18" t="n"/>
       <c r="P198" s="18" t="n"/>
-      <c r="Q198" s="18" t="inlineStr"/>
+      <c r="Q198" s="18" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="18" t="inlineStr">
@@ -15978,7 +16080,7 @@
       </c>
       <c r="O199" s="18" t="n"/>
       <c r="P199" s="18" t="n"/>
-      <c r="Q199" s="18" t="inlineStr"/>
+      <c r="Q199" s="18" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="18" t="inlineStr">
@@ -16045,7 +16147,7 @@
       </c>
       <c r="O200" s="18" t="n"/>
       <c r="P200" s="18" t="n"/>
-      <c r="Q200" s="18" t="inlineStr"/>
+      <c r="Q200" s="18" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="18" t="inlineStr">
@@ -16112,7 +16214,7 @@
       </c>
       <c r="O201" s="18" t="n"/>
       <c r="P201" s="18" t="n"/>
-      <c r="Q201" s="18" t="inlineStr"/>
+      <c r="Q201" s="18" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="18" t="inlineStr">
@@ -16179,7 +16281,7 @@
       </c>
       <c r="O202" s="18" t="n"/>
       <c r="P202" s="18" t="n"/>
-      <c r="Q202" s="18" t="inlineStr"/>
+      <c r="Q202" s="18" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="18" t="inlineStr">
@@ -16246,7 +16348,7 @@
       </c>
       <c r="O203" s="18" t="n"/>
       <c r="P203" s="18" t="n"/>
-      <c r="Q203" s="18" t="inlineStr"/>
+      <c r="Q203" s="18" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="18" t="inlineStr">
@@ -16313,7 +16415,7 @@
       </c>
       <c r="O204" s="18" t="n"/>
       <c r="P204" s="18" t="n"/>
-      <c r="Q204" s="18" t="inlineStr"/>
+      <c r="Q204" s="18" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="18" t="inlineStr">
@@ -17587,7 +17689,7 @@
       </c>
       <c r="O222" s="18" t="n"/>
       <c r="P222" s="18" t="n"/>
-      <c r="Q222" s="18" t="inlineStr"/>
+      <c r="Q222" s="18" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="18" t="inlineStr">
@@ -17654,7 +17756,7 @@
       </c>
       <c r="O223" s="18" t="n"/>
       <c r="P223" s="18" t="n"/>
-      <c r="Q223" s="18" t="inlineStr"/>
+      <c r="Q223" s="18" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="18" t="inlineStr">
@@ -17721,7 +17823,7 @@
       </c>
       <c r="O224" s="18" t="n"/>
       <c r="P224" s="18" t="n"/>
-      <c r="Q224" s="18" t="inlineStr"/>
+      <c r="Q224" s="18" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="18" t="inlineStr">
@@ -17788,7 +17890,7 @@
       </c>
       <c r="O225" s="18" t="n"/>
       <c r="P225" s="18" t="n"/>
-      <c r="Q225" s="18" t="inlineStr"/>
+      <c r="Q225" s="18" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="18" t="inlineStr">
@@ -17855,7 +17957,7 @@
       </c>
       <c r="O226" s="18" t="n"/>
       <c r="P226" s="18" t="n"/>
-      <c r="Q226" s="18" t="inlineStr"/>
+      <c r="Q226" s="18" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="18" t="inlineStr">
@@ -18703,7 +18805,7 @@
       </c>
       <c r="O238" s="18" t="n"/>
       <c r="P238" s="18" t="n"/>
-      <c r="Q238" s="18" t="inlineStr"/>
+      <c r="Q238" s="18" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="18" t="inlineStr">
@@ -18770,7 +18872,7 @@
       </c>
       <c r="O239" s="18" t="n"/>
       <c r="P239" s="18" t="n"/>
-      <c r="Q239" s="18" t="inlineStr"/>
+      <c r="Q239" s="18" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="18" t="inlineStr">
@@ -18837,7 +18939,7 @@
       </c>
       <c r="O240" s="18" t="n"/>
       <c r="P240" s="18" t="n"/>
-      <c r="Q240" s="18" t="inlineStr"/>
+      <c r="Q240" s="18" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="18" t="inlineStr">
@@ -18904,7 +19006,7 @@
       </c>
       <c r="O241" s="18" t="n"/>
       <c r="P241" s="18" t="n"/>
-      <c r="Q241" s="18" t="inlineStr"/>
+      <c r="Q241" s="18" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="18" t="inlineStr">
@@ -18971,7 +19073,7 @@
       </c>
       <c r="O242" s="18" t="n"/>
       <c r="P242" s="18" t="n"/>
-      <c r="Q242" s="18" t="inlineStr"/>
+      <c r="Q242" s="18" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="18" t="inlineStr">
@@ -19038,7 +19140,7 @@
       </c>
       <c r="O243" s="18" t="n"/>
       <c r="P243" s="18" t="n"/>
-      <c r="Q243" s="18" t="inlineStr"/>
+      <c r="Q243" s="18" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="18" t="inlineStr">
@@ -19105,7 +19207,7 @@
       </c>
       <c r="O244" s="18" t="n"/>
       <c r="P244" s="18" t="n"/>
-      <c r="Q244" s="18" t="inlineStr"/>
+      <c r="Q244" s="18" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="18" t="inlineStr">
@@ -19172,7 +19274,7 @@
       </c>
       <c r="O245" s="18" t="n"/>
       <c r="P245" s="18" t="n"/>
-      <c r="Q245" s="18" t="inlineStr"/>
+      <c r="Q245" s="18" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="18" t="inlineStr">
@@ -19239,7 +19341,7 @@
       </c>
       <c r="O246" s="18" t="n"/>
       <c r="P246" s="18" t="n"/>
-      <c r="Q246" s="18" t="inlineStr"/>
+      <c r="Q246" s="18" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="18" t="inlineStr">
@@ -19306,7 +19408,7 @@
       </c>
       <c r="O247" s="18" t="n"/>
       <c r="P247" s="18" t="n"/>
-      <c r="Q247" s="18" t="inlineStr"/>
+      <c r="Q247" s="18" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="18" t="inlineStr">
@@ -19373,7 +19475,7 @@
       </c>
       <c r="O248" s="18" t="n"/>
       <c r="P248" s="18" t="n"/>
-      <c r="Q248" s="18" t="inlineStr"/>
+      <c r="Q248" s="18" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="18" t="inlineStr">
@@ -19440,7 +19542,7 @@
       </c>
       <c r="O249" s="18" t="n"/>
       <c r="P249" s="18" t="n"/>
-      <c r="Q249" s="18" t="inlineStr"/>
+      <c r="Q249" s="18" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="18" t="inlineStr">
@@ -19507,7 +19609,7 @@
       </c>
       <c r="O250" s="18" t="n"/>
       <c r="P250" s="18" t="n"/>
-      <c r="Q250" s="18" t="inlineStr"/>
+      <c r="Q250" s="18" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="18" t="inlineStr">
@@ -19574,7 +19676,7 @@
       </c>
       <c r="O251" s="18" t="n"/>
       <c r="P251" s="18" t="n"/>
-      <c r="Q251" s="18" t="inlineStr"/>
+      <c r="Q251" s="18" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="18" t="inlineStr">
@@ -19641,7 +19743,7 @@
       </c>
       <c r="O252" s="18" t="n"/>
       <c r="P252" s="18" t="n"/>
-      <c r="Q252" s="18" t="inlineStr"/>
+      <c r="Q252" s="18" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="18" t="inlineStr">
@@ -19708,7 +19810,7 @@
       </c>
       <c r="O253" s="18" t="n"/>
       <c r="P253" s="18" t="n"/>
-      <c r="Q253" s="18" t="inlineStr"/>
+      <c r="Q253" s="18" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="18" t="inlineStr">
@@ -19775,7 +19877,7 @@
       </c>
       <c r="O254" s="18" t="n"/>
       <c r="P254" s="18" t="n"/>
-      <c r="Q254" s="18" t="inlineStr"/>
+      <c r="Q254" s="18" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="18" t="inlineStr">
@@ -19842,7 +19944,7 @@
       </c>
       <c r="O255" s="18" t="n"/>
       <c r="P255" s="18" t="n"/>
-      <c r="Q255" s="18" t="inlineStr"/>
+      <c r="Q255" s="18" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="18" t="inlineStr">
@@ -19909,7 +20011,7 @@
       </c>
       <c r="O256" s="18" t="n"/>
       <c r="P256" s="18" t="n"/>
-      <c r="Q256" s="18" t="inlineStr"/>
+      <c r="Q256" s="18" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="18" t="inlineStr">
@@ -19976,7 +20078,7 @@
       </c>
       <c r="O257" s="18" t="n"/>
       <c r="P257" s="18" t="n"/>
-      <c r="Q257" s="18" t="inlineStr"/>
+      <c r="Q257" s="18" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="18" t="inlineStr">
@@ -20043,7 +20145,7 @@
       </c>
       <c r="O258" s="18" t="n"/>
       <c r="P258" s="18" t="n"/>
-      <c r="Q258" s="18" t="inlineStr"/>
+      <c r="Q258" s="18" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="18" t="inlineStr">
@@ -20110,7 +20212,7 @@
       </c>
       <c r="O259" s="18" t="n"/>
       <c r="P259" s="18" t="n"/>
-      <c r="Q259" s="18" t="inlineStr"/>
+      <c r="Q259" s="18" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="18" t="inlineStr">
@@ -20177,7 +20279,7 @@
       </c>
       <c r="O260" s="18" t="n"/>
       <c r="P260" s="18" t="n"/>
-      <c r="Q260" s="18" t="inlineStr"/>
+      <c r="Q260" s="18" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="18" t="inlineStr">
@@ -20244,7 +20346,7 @@
       </c>
       <c r="O261" s="18" t="n"/>
       <c r="P261" s="18" t="n"/>
-      <c r="Q261" s="18" t="inlineStr"/>
+      <c r="Q261" s="18" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="18" t="inlineStr">
@@ -20311,7 +20413,7 @@
       </c>
       <c r="O262" s="18" t="n"/>
       <c r="P262" s="18" t="n"/>
-      <c r="Q262" s="18" t="inlineStr"/>
+      <c r="Q262" s="18" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="18" t="inlineStr">
@@ -20449,7 +20551,7 @@
       </c>
       <c r="O264" s="18" t="n"/>
       <c r="P264" s="18" t="n"/>
-      <c r="Q264" s="18" t="inlineStr"/>
+      <c r="Q264" s="18" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="18" t="inlineStr">
@@ -20516,7 +20618,7 @@
       </c>
       <c r="O265" s="18" t="n"/>
       <c r="P265" s="18" t="n"/>
-      <c r="Q265" s="18" t="inlineStr"/>
+      <c r="Q265" s="18" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="18" t="inlineStr">
@@ -20583,7 +20685,7 @@
       </c>
       <c r="O266" s="18" t="n"/>
       <c r="P266" s="18" t="n"/>
-      <c r="Q266" s="18" t="inlineStr"/>
+      <c r="Q266" s="18" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="18" t="inlineStr">
@@ -20650,7 +20752,7 @@
       </c>
       <c r="O267" s="18" t="n"/>
       <c r="P267" s="18" t="n"/>
-      <c r="Q267" s="18" t="inlineStr"/>
+      <c r="Q267" s="18" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="18" t="inlineStr">
@@ -20717,7 +20819,7 @@
       </c>
       <c r="O268" s="18" t="n"/>
       <c r="P268" s="18" t="n"/>
-      <c r="Q268" s="18" t="inlineStr"/>
+      <c r="Q268" s="18" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="18" t="inlineStr">
@@ -20784,7 +20886,7 @@
       </c>
       <c r="O269" s="18" t="n"/>
       <c r="P269" s="18" t="n"/>
-      <c r="Q269" s="18" t="inlineStr"/>
+      <c r="Q269" s="18" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="18" t="inlineStr">
@@ -20851,7 +20953,7 @@
       </c>
       <c r="O270" s="18" t="n"/>
       <c r="P270" s="18" t="n"/>
-      <c r="Q270" s="18" t="inlineStr"/>
+      <c r="Q270" s="18" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="18" t="inlineStr">
@@ -20918,7 +21020,7 @@
       </c>
       <c r="O271" s="18" t="n"/>
       <c r="P271" s="18" t="n"/>
-      <c r="Q271" s="18" t="inlineStr"/>
+      <c r="Q271" s="18" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="18" t="inlineStr">
@@ -20985,7 +21087,7 @@
       </c>
       <c r="O272" s="18" t="n"/>
       <c r="P272" s="18" t="n"/>
-      <c r="Q272" s="18" t="inlineStr"/>
+      <c r="Q272" s="18" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="18" t="inlineStr">
@@ -21052,7 +21154,7 @@
       </c>
       <c r="O273" s="18" t="n"/>
       <c r="P273" s="18" t="n"/>
-      <c r="Q273" s="18" t="inlineStr"/>
+      <c r="Q273" s="18" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="18" t="inlineStr">
@@ -21119,7 +21221,7 @@
       </c>
       <c r="O274" s="18" t="n"/>
       <c r="P274" s="18" t="n"/>
-      <c r="Q274" s="18" t="inlineStr"/>
+      <c r="Q274" s="18" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="18" t="inlineStr">
@@ -21186,7 +21288,7 @@
       </c>
       <c r="O275" s="18" t="n"/>
       <c r="P275" s="18" t="n"/>
-      <c r="Q275" s="18" t="inlineStr"/>
+      <c r="Q275" s="18" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="18" t="inlineStr">
@@ -21253,7 +21355,7 @@
       </c>
       <c r="O276" s="18" t="n"/>
       <c r="P276" s="18" t="n"/>
-      <c r="Q276" s="18" t="inlineStr"/>
+      <c r="Q276" s="18" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="18" t="inlineStr">
@@ -21320,7 +21422,7 @@
       </c>
       <c r="O277" s="18" t="n"/>
       <c r="P277" s="18" t="n"/>
-      <c r="Q277" s="18" t="inlineStr"/>
+      <c r="Q277" s="18" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="18" t="inlineStr">
@@ -21387,7 +21489,7 @@
       </c>
       <c r="O278" s="18" t="n"/>
       <c r="P278" s="18" t="n"/>
-      <c r="Q278" s="18" t="inlineStr"/>
+      <c r="Q278" s="18" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="18" t="inlineStr">
@@ -21454,7 +21556,7 @@
       </c>
       <c r="O279" s="18" t="n"/>
       <c r="P279" s="18" t="n"/>
-      <c r="Q279" s="18" t="inlineStr"/>
+      <c r="Q279" s="18" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="18" t="inlineStr">
@@ -21521,7 +21623,7 @@
       </c>
       <c r="O280" s="18" t="n"/>
       <c r="P280" s="18" t="n"/>
-      <c r="Q280" s="18" t="inlineStr"/>
+      <c r="Q280" s="18" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="18" t="inlineStr">
@@ -21588,7 +21690,7 @@
       </c>
       <c r="O281" s="18" t="n"/>
       <c r="P281" s="18" t="n"/>
-      <c r="Q281" s="18" t="inlineStr"/>
+      <c r="Q281" s="18" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="18" t="inlineStr">
@@ -21655,7 +21757,7 @@
       </c>
       <c r="O282" s="18" t="n"/>
       <c r="P282" s="18" t="n"/>
-      <c r="Q282" s="18" t="inlineStr"/>
+      <c r="Q282" s="18" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="18" t="inlineStr">
@@ -21722,7 +21824,7 @@
       </c>
       <c r="O283" s="18" t="n"/>
       <c r="P283" s="18" t="n"/>
-      <c r="Q283" s="18" t="inlineStr"/>
+      <c r="Q283" s="18" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="18" t="inlineStr">
@@ -21789,7 +21891,7 @@
       </c>
       <c r="O284" s="18" t="n"/>
       <c r="P284" s="18" t="n"/>
-      <c r="Q284" s="18" t="inlineStr"/>
+      <c r="Q284" s="18" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="18" t="inlineStr">
@@ -21856,7 +21958,7 @@
       </c>
       <c r="O285" s="18" t="n"/>
       <c r="P285" s="18" t="n"/>
-      <c r="Q285" s="18" t="inlineStr"/>
+      <c r="Q285" s="18" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="18" t="inlineStr">
@@ -21923,7 +22025,7 @@
       </c>
       <c r="O286" s="18" t="n"/>
       <c r="P286" s="18" t="n"/>
-      <c r="Q286" s="18" t="inlineStr"/>
+      <c r="Q286" s="18" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="18" t="inlineStr">
@@ -21990,7 +22092,7 @@
       </c>
       <c r="O287" s="18" t="n"/>
       <c r="P287" s="18" t="n"/>
-      <c r="Q287" s="18" t="inlineStr"/>
+      <c r="Q287" s="18" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="18" t="inlineStr">
@@ -22057,7 +22159,7 @@
       </c>
       <c r="O288" s="18" t="n"/>
       <c r="P288" s="18" t="n"/>
-      <c r="Q288" s="18" t="inlineStr"/>
+      <c r="Q288" s="18" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="18" t="inlineStr">
@@ -22195,7 +22297,7 @@
       </c>
       <c r="O290" s="18" t="n"/>
       <c r="P290" s="18" t="n"/>
-      <c r="Q290" s="18" t="inlineStr"/>
+      <c r="Q290" s="18" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="18" t="inlineStr">
@@ -22262,7 +22364,7 @@
       </c>
       <c r="O291" s="18" t="n"/>
       <c r="P291" s="18" t="n"/>
-      <c r="Q291" s="18" t="inlineStr"/>
+      <c r="Q291" s="18" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="18" t="inlineStr">
@@ -22329,7 +22431,7 @@
       </c>
       <c r="O292" s="18" t="n"/>
       <c r="P292" s="18" t="n"/>
-      <c r="Q292" s="18" t="inlineStr"/>
+      <c r="Q292" s="18" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="18" t="inlineStr">
@@ -22396,7 +22498,7 @@
       </c>
       <c r="O293" s="18" t="n"/>
       <c r="P293" s="18" t="n"/>
-      <c r="Q293" s="18" t="inlineStr"/>
+      <c r="Q293" s="18" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="18" t="inlineStr">
@@ -22463,7 +22565,7 @@
       </c>
       <c r="O294" s="18" t="n"/>
       <c r="P294" s="18" t="n"/>
-      <c r="Q294" s="18" t="inlineStr"/>
+      <c r="Q294" s="18" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="18" t="inlineStr">
@@ -22530,7 +22632,7 @@
       </c>
       <c r="O295" s="18" t="n"/>
       <c r="P295" s="18" t="n"/>
-      <c r="Q295" s="18" t="inlineStr"/>
+      <c r="Q295" s="18" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="18" t="inlineStr">
@@ -22597,7 +22699,7 @@
       </c>
       <c r="O296" s="18" t="n"/>
       <c r="P296" s="18" t="n"/>
-      <c r="Q296" s="18" t="inlineStr"/>
+      <c r="Q296" s="18" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="18" t="inlineStr">
@@ -22664,7 +22766,7 @@
       </c>
       <c r="O297" s="18" t="n"/>
       <c r="P297" s="18" t="n"/>
-      <c r="Q297" s="18" t="inlineStr"/>
+      <c r="Q297" s="18" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="18" t="inlineStr">
@@ -22731,7 +22833,7 @@
       </c>
       <c r="O298" s="18" t="n"/>
       <c r="P298" s="18" t="n"/>
-      <c r="Q298" s="18" t="inlineStr"/>
+      <c r="Q298" s="18" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="18" t="inlineStr">
@@ -22798,7 +22900,7 @@
       </c>
       <c r="O299" s="18" t="n"/>
       <c r="P299" s="18" t="n"/>
-      <c r="Q299" s="18" t="inlineStr"/>
+      <c r="Q299" s="18" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="18" t="inlineStr">
@@ -22865,7 +22967,7 @@
       </c>
       <c r="O300" s="18" t="n"/>
       <c r="P300" s="18" t="n"/>
-      <c r="Q300" s="18" t="inlineStr"/>
+      <c r="Q300" s="18" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="18" t="inlineStr">
@@ -22932,7 +23034,7 @@
       </c>
       <c r="O301" s="18" t="n"/>
       <c r="P301" s="18" t="n"/>
-      <c r="Q301" s="18" t="inlineStr"/>
+      <c r="Q301" s="18" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="18" t="inlineStr">
@@ -22999,7 +23101,7 @@
       </c>
       <c r="O302" s="18" t="n"/>
       <c r="P302" s="18" t="n"/>
-      <c r="Q302" s="18" t="inlineStr"/>
+      <c r="Q302" s="18" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="18" t="inlineStr">
@@ -23066,7 +23168,7 @@
       </c>
       <c r="O303" s="18" t="n"/>
       <c r="P303" s="18" t="n"/>
-      <c r="Q303" s="18" t="inlineStr"/>
+      <c r="Q303" s="18" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="18" t="inlineStr">
@@ -23133,7 +23235,7 @@
       </c>
       <c r="O304" s="18" t="n"/>
       <c r="P304" s="18" t="n"/>
-      <c r="Q304" s="18" t="inlineStr"/>
+      <c r="Q304" s="18" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="18" t="inlineStr">
@@ -23200,7 +23302,7 @@
       </c>
       <c r="O305" s="18" t="n"/>
       <c r="P305" s="18" t="n"/>
-      <c r="Q305" s="18" t="inlineStr"/>
+      <c r="Q305" s="18" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="18" t="inlineStr">
@@ -23267,7 +23369,7 @@
       </c>
       <c r="O306" s="18" t="n"/>
       <c r="P306" s="18" t="n"/>
-      <c r="Q306" s="18" t="inlineStr"/>
+      <c r="Q306" s="18" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="18" t="inlineStr">
@@ -23334,7 +23436,7 @@
       </c>
       <c r="O307" s="18" t="n"/>
       <c r="P307" s="18" t="n"/>
-      <c r="Q307" s="18" t="inlineStr"/>
+      <c r="Q307" s="18" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="18" t="inlineStr">
@@ -23401,7 +23503,7 @@
       </c>
       <c r="O308" s="18" t="n"/>
       <c r="P308" s="18" t="n"/>
-      <c r="Q308" s="18" t="inlineStr"/>
+      <c r="Q308" s="18" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="18" t="inlineStr">
@@ -23468,7 +23570,7 @@
       </c>
       <c r="O309" s="18" t="n"/>
       <c r="P309" s="18" t="n"/>
-      <c r="Q309" s="18" t="inlineStr"/>
+      <c r="Q309" s="18" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="18" t="inlineStr">
@@ -23535,7 +23637,7 @@
       </c>
       <c r="O310" s="18" t="n"/>
       <c r="P310" s="18" t="n"/>
-      <c r="Q310" s="18" t="inlineStr"/>
+      <c r="Q310" s="18" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="18" t="inlineStr">
@@ -23602,7 +23704,7 @@
       </c>
       <c r="O311" s="18" t="n"/>
       <c r="P311" s="18" t="n"/>
-      <c r="Q311" s="18" t="inlineStr"/>
+      <c r="Q311" s="18" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="18" t="inlineStr">
@@ -23669,7 +23771,7 @@
       </c>
       <c r="O312" s="18" t="n"/>
       <c r="P312" s="18" t="n"/>
-      <c r="Q312" s="18" t="inlineStr"/>
+      <c r="Q312" s="18" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="18" t="inlineStr">
@@ -23736,7 +23838,7 @@
       </c>
       <c r="O313" s="18" t="n"/>
       <c r="P313" s="18" t="n"/>
-      <c r="Q313" s="18" t="inlineStr"/>
+      <c r="Q313" s="18" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="18" t="inlineStr">
@@ -23803,7 +23905,7 @@
       </c>
       <c r="O314" s="18" t="n"/>
       <c r="P314" s="18" t="n"/>
-      <c r="Q314" s="18" t="inlineStr"/>
+      <c r="Q314" s="18" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="18" t="inlineStr">
@@ -23870,7 +23972,7 @@
       </c>
       <c r="O315" s="18" t="n"/>
       <c r="P315" s="18" t="n"/>
-      <c r="Q315" s="18" t="inlineStr"/>
+      <c r="Q315" s="18" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="18" t="inlineStr">
@@ -23937,7 +24039,7 @@
       </c>
       <c r="O316" s="18" t="n"/>
       <c r="P316" s="18" t="n"/>
-      <c r="Q316" s="18" t="inlineStr"/>
+      <c r="Q316" s="18" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="18" t="inlineStr">
@@ -24004,7 +24106,7 @@
       </c>
       <c r="O317" s="18" t="n"/>
       <c r="P317" s="18" t="n"/>
-      <c r="Q317" s="18" t="inlineStr"/>
+      <c r="Q317" s="18" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="18" t="inlineStr">
@@ -24071,7 +24173,7 @@
       </c>
       <c r="O318" s="18" t="n"/>
       <c r="P318" s="18" t="n"/>
-      <c r="Q318" s="18" t="inlineStr"/>
+      <c r="Q318" s="18" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="18" t="inlineStr">
@@ -24138,7 +24240,7 @@
       </c>
       <c r="O319" s="18" t="n"/>
       <c r="P319" s="18" t="n"/>
-      <c r="Q319" s="18" t="inlineStr"/>
+      <c r="Q319" s="18" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="18" t="inlineStr">
@@ -24205,7 +24307,7 @@
       </c>
       <c r="O320" s="18" t="n"/>
       <c r="P320" s="18" t="n"/>
-      <c r="Q320" s="18" t="inlineStr"/>
+      <c r="Q320" s="18" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="18" t="inlineStr">
@@ -24272,7 +24374,7 @@
       </c>
       <c r="O321" s="18" t="n"/>
       <c r="P321" s="18" t="n"/>
-      <c r="Q321" s="18" t="inlineStr"/>
+      <c r="Q321" s="18" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="18" t="inlineStr">
@@ -24339,7 +24441,7 @@
       </c>
       <c r="O322" s="18" t="n"/>
       <c r="P322" s="18" t="n"/>
-      <c r="Q322" s="18" t="inlineStr"/>
+      <c r="Q322" s="18" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="18" t="inlineStr">
@@ -24406,7 +24508,7 @@
       </c>
       <c r="O323" s="18" t="n"/>
       <c r="P323" s="18" t="n"/>
-      <c r="Q323" s="18" t="inlineStr"/>
+      <c r="Q323" s="18" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="18" t="inlineStr">
@@ -24473,7 +24575,7 @@
       </c>
       <c r="O324" s="18" t="n"/>
       <c r="P324" s="18" t="n"/>
-      <c r="Q324" s="18" t="inlineStr"/>
+      <c r="Q324" s="18" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="18" t="inlineStr">
@@ -24540,7 +24642,7 @@
       </c>
       <c r="O325" s="18" t="n"/>
       <c r="P325" s="18" t="n"/>
-      <c r="Q325" s="18" t="inlineStr"/>
+      <c r="Q325" s="18" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="18" t="inlineStr">
@@ -24607,7 +24709,7 @@
       </c>
       <c r="O326" s="18" t="n"/>
       <c r="P326" s="18" t="n"/>
-      <c r="Q326" s="18" t="inlineStr"/>
+      <c r="Q326" s="18" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="18" t="inlineStr">
@@ -24674,7 +24776,7 @@
       </c>
       <c r="O327" s="18" t="n"/>
       <c r="P327" s="18" t="n"/>
-      <c r="Q327" s="18" t="inlineStr"/>
+      <c r="Q327" s="18" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="18" t="inlineStr">
@@ -24741,7 +24843,7 @@
       </c>
       <c r="O328" s="18" t="n"/>
       <c r="P328" s="18" t="n"/>
-      <c r="Q328" s="18" t="inlineStr"/>
+      <c r="Q328" s="18" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="18" t="inlineStr">
@@ -24808,7 +24910,7 @@
       </c>
       <c r="O329" s="18" t="n"/>
       <c r="P329" s="18" t="n"/>
-      <c r="Q329" s="18" t="inlineStr"/>
+      <c r="Q329" s="18" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="18" t="inlineStr">
@@ -24875,7 +24977,7 @@
       </c>
       <c r="O330" s="18" t="n"/>
       <c r="P330" s="18" t="n"/>
-      <c r="Q330" s="18" t="inlineStr"/>
+      <c r="Q330" s="18" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="18" t="inlineStr">
@@ -24942,7 +25044,7 @@
       </c>
       <c r="O331" s="18" t="n"/>
       <c r="P331" s="18" t="n"/>
-      <c r="Q331" s="18" t="inlineStr"/>
+      <c r="Q331" s="18" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="18" t="inlineStr">
@@ -25009,7 +25111,7 @@
       </c>
       <c r="O332" s="18" t="n"/>
       <c r="P332" s="18" t="n"/>
-      <c r="Q332" s="18" t="inlineStr"/>
+      <c r="Q332" s="18" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="18" t="inlineStr">
@@ -25076,7 +25178,7 @@
       </c>
       <c r="O333" s="18" t="n"/>
       <c r="P333" s="18" t="n"/>
-      <c r="Q333" s="18" t="inlineStr"/>
+      <c r="Q333" s="18" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="18" t="inlineStr">
@@ -25214,7 +25316,7 @@
       </c>
       <c r="O335" s="18" t="n"/>
       <c r="P335" s="18" t="n"/>
-      <c r="Q335" s="18" t="inlineStr"/>
+      <c r="Q335" s="18" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q335"/>

</xml_diff>

<commit_message>
Add interface specification documents for all ERP interfaces
17 ISDs (one per interface ID in scope §D.4.2) plus ISD-00 common
conventions: SAP ECC/S4 and Oracle EBS/Fusion realisation, canonical
message definition, field mapping, processing rules, error codes,
test scenarios and open points. Scope §D.4 and README link the ISDs;
RTM interface rows default their Design Reference to the ISD.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/rtm/AstraWMS_RTM.xlsx
+++ b/docs/rtm/AstraWMS_RTM.xlsx
@@ -16459,7 +16459,11 @@
         </is>
       </c>
       <c r="I205" s="18" t="n"/>
-      <c r="J205" s="18" t="n"/>
+      <c r="J205" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-IB-001.md</t>
+        </is>
+      </c>
       <c r="K205" s="18" t="inlineStr">
         <is>
           <t>TC-IF-IB-001-01</t>
@@ -16530,7 +16534,11 @@
         </is>
       </c>
       <c r="I206" s="18" t="n"/>
-      <c r="J206" s="18" t="n"/>
+      <c r="J206" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-IB-002.md</t>
+        </is>
+      </c>
       <c r="K206" s="18" t="inlineStr">
         <is>
           <t>TC-IF-IB-002-01</t>
@@ -16601,7 +16609,11 @@
         </is>
       </c>
       <c r="I207" s="18" t="n"/>
-      <c r="J207" s="18" t="n"/>
+      <c r="J207" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-INV-001.md</t>
+        </is>
+      </c>
       <c r="K207" s="18" t="inlineStr">
         <is>
           <t>TC-IF-INV-001-01</t>
@@ -16672,7 +16684,11 @@
         </is>
       </c>
       <c r="I208" s="18" t="n"/>
-      <c r="J208" s="18" t="n"/>
+      <c r="J208" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-INV-002.md</t>
+        </is>
+      </c>
       <c r="K208" s="18" t="inlineStr">
         <is>
           <t>TC-IF-INV-002-01</t>
@@ -16743,7 +16759,11 @@
         </is>
       </c>
       <c r="I209" s="18" t="n"/>
-      <c r="J209" s="18" t="n"/>
+      <c r="J209" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-INV-003.md</t>
+        </is>
+      </c>
       <c r="K209" s="18" t="inlineStr">
         <is>
           <t>TC-IF-INV-003-01</t>
@@ -16814,7 +16834,11 @@
         </is>
       </c>
       <c r="I210" s="18" t="n"/>
-      <c r="J210" s="18" t="n"/>
+      <c r="J210" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-INV-004.md</t>
+        </is>
+      </c>
       <c r="K210" s="18" t="inlineStr">
         <is>
           <t>TC-IF-INV-004-01</t>
@@ -16885,7 +16909,11 @@
         </is>
       </c>
       <c r="I211" s="18" t="n"/>
-      <c r="J211" s="18" t="n"/>
+      <c r="J211" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-KIT-001.md</t>
+        </is>
+      </c>
       <c r="K211" s="18" t="inlineStr">
         <is>
           <t>TC-IF-KIT-001-01</t>
@@ -16956,7 +16984,11 @@
         </is>
       </c>
       <c r="I212" s="18" t="n"/>
-      <c r="J212" s="18" t="n"/>
+      <c r="J212" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-MD-001.md</t>
+        </is>
+      </c>
       <c r="K212" s="18" t="inlineStr">
         <is>
           <t>TC-IF-MD-001-01</t>
@@ -17027,7 +17059,11 @@
         </is>
       </c>
       <c r="I213" s="18" t="n"/>
-      <c r="J213" s="18" t="n"/>
+      <c r="J213" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-MD-002.md</t>
+        </is>
+      </c>
       <c r="K213" s="18" t="inlineStr">
         <is>
           <t>TC-IF-MD-002-01</t>
@@ -17098,7 +17134,11 @@
         </is>
       </c>
       <c r="I214" s="18" t="n"/>
-      <c r="J214" s="18" t="n"/>
+      <c r="J214" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-MD-003.md</t>
+        </is>
+      </c>
       <c r="K214" s="18" t="inlineStr">
         <is>
           <t>TC-IF-MD-003-01</t>
@@ -17169,7 +17209,11 @@
         </is>
       </c>
       <c r="I215" s="18" t="n"/>
-      <c r="J215" s="18" t="n"/>
+      <c r="J215" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-MD-004.md</t>
+        </is>
+      </c>
       <c r="K215" s="18" t="inlineStr">
         <is>
           <t>TC-IF-MD-004-01</t>
@@ -17240,7 +17284,11 @@
         </is>
       </c>
       <c r="I216" s="18" t="n"/>
-      <c r="J216" s="18" t="n"/>
+      <c r="J216" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-OB-001.md</t>
+        </is>
+      </c>
       <c r="K216" s="18" t="inlineStr">
         <is>
           <t>TC-IF-OB-001-01</t>
@@ -17311,7 +17359,11 @@
         </is>
       </c>
       <c r="I217" s="18" t="n"/>
-      <c r="J217" s="18" t="n"/>
+      <c r="J217" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-OB-002.md</t>
+        </is>
+      </c>
       <c r="K217" s="18" t="inlineStr">
         <is>
           <t>TC-IF-OB-002-01</t>
@@ -17382,7 +17434,11 @@
         </is>
       </c>
       <c r="I218" s="18" t="n"/>
-      <c r="J218" s="18" t="n"/>
+      <c r="J218" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-OB-003.md</t>
+        </is>
+      </c>
       <c r="K218" s="18" t="inlineStr">
         <is>
           <t>TC-IF-OB-003-01</t>
@@ -17453,7 +17509,11 @@
         </is>
       </c>
       <c r="I219" s="18" t="n"/>
-      <c r="J219" s="18" t="n"/>
+      <c r="J219" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-OB-004.md</t>
+        </is>
+      </c>
       <c r="K219" s="18" t="inlineStr">
         <is>
           <t>TC-IF-OB-004-01</t>
@@ -17524,7 +17584,11 @@
         </is>
       </c>
       <c r="I220" s="18" t="n"/>
-      <c r="J220" s="18" t="n"/>
+      <c r="J220" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-RET-001.md</t>
+        </is>
+      </c>
       <c r="K220" s="18" t="inlineStr">
         <is>
           <t>TC-IF-RET-001-01</t>
@@ -17595,7 +17659,11 @@
         </is>
       </c>
       <c r="I221" s="18" t="n"/>
-      <c r="J221" s="18" t="n"/>
+      <c r="J221" s="18" t="inlineStr">
+        <is>
+          <t>docs/isd/IF-RET-002.md</t>
+        </is>
+      </c>
       <c r="K221" s="18" t="inlineStr">
         <is>
           <t>TC-IF-RET-002-01</t>

</xml_diff>